<commit_message>
adding cumulative macroeconomic impacts.
</commit_message>
<xml_diff>
--- a/tables_used_in_main/Economic_indicator.xlsx
+++ b/tables_used_in_main/Economic_indicator.xlsx
@@ -5,25 +5,39 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shiya/Desktop/Model/ScenarioMIP/LN_Marker/output/table/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shiya/Desktop/Model/ScenarioMIP/LN_Marker/tables_used_in_main/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40D6C9FE-1F70-7E47-8CE3-1785E70DE453}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1556F766-8202-5C47-9212-0DAB11F68132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
+    <sheet name="compare with the relative Mediu" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$A$1:$Y$174</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1409" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1594" uniqueCount="68">
   <si>
     <t>Model</t>
   </si>
@@ -222,12 +236,18 @@
   <si>
     <t>Consumption change from SSP2_M</t>
   </si>
+  <si>
+    <t>GDP change from Medium</t>
+  </si>
+  <si>
+    <t>Consumption change from Medium</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -242,8 +262,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="8" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="6" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -268,8 +302,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -301,15 +341,45 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
@@ -320,6 +390,30 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -847,7 +941,7 @@
       <c r="W3">
         <v>719.8664</v>
       </c>
-      <c r="X3" s="3">
+      <c r="X3">
         <v>713.50340000000006</v>
       </c>
       <c r="Y3" s="1">
@@ -855,79 +949,79 @@
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="I4" s="5">
-        <v>0</v>
-      </c>
-      <c r="J4" s="5">
-        <v>0</v>
-      </c>
-      <c r="K4" s="5">
+      <c r="I4" s="4">
+        <v>0</v>
+      </c>
+      <c r="J4" s="4">
+        <v>0</v>
+      </c>
+      <c r="K4" s="4">
         <v>5.5458999999999996</v>
       </c>
-      <c r="L4" s="5">
+      <c r="L4" s="4">
         <v>4.9405000000000001</v>
       </c>
-      <c r="M4" s="5">
+      <c r="M4" s="4">
         <v>71.909400000000005</v>
       </c>
-      <c r="N4" s="5">
+      <c r="N4" s="4">
         <v>107.1816</v>
       </c>
-      <c r="O4" s="5">
+      <c r="O4" s="4">
         <v>144.29230000000001</v>
       </c>
-      <c r="P4" s="5">
+      <c r="P4" s="4">
         <v>202.06010000000001</v>
       </c>
-      <c r="Q4" s="5">
+      <c r="Q4" s="4">
         <v>322.90879999999999</v>
       </c>
-      <c r="R4" s="5">
+      <c r="R4" s="4">
         <v>593.98360000000002</v>
       </c>
-      <c r="S4" s="5">
+      <c r="S4" s="4">
         <v>713.03250000000003</v>
       </c>
-      <c r="T4" s="5">
+      <c r="T4" s="4">
         <v>716.11850000000004</v>
       </c>
-      <c r="U4" s="5">
+      <c r="U4" s="4">
         <v>773.36220000000003</v>
       </c>
-      <c r="V4" s="5">
+      <c r="V4" s="4">
         <v>805.63239999999996</v>
       </c>
-      <c r="W4" s="5">
+      <c r="W4" s="4">
         <v>716.91589999999997</v>
       </c>
-      <c r="X4" s="5">
+      <c r="X4" s="4">
         <v>714.26390000000004</v>
       </c>
-      <c r="Y4" s="5">
+      <c r="Y4" s="4">
         <v>718.51279999999997</v>
       </c>
     </row>
@@ -1155,7 +1249,7 @@
       <c r="W7">
         <v>415.34249999999997</v>
       </c>
-      <c r="X7" s="3">
+      <c r="X7">
         <v>435.02510000000001</v>
       </c>
       <c r="Y7" s="1">
@@ -1163,361 +1257,361 @@
       </c>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H8" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I8" s="4">
-        <v>0</v>
-      </c>
-      <c r="J8" s="4">
+      <c r="I8" s="3">
+        <v>0</v>
+      </c>
+      <c r="J8" s="3">
         <v>33.540309912292102</v>
       </c>
-      <c r="K8" s="4">
+      <c r="K8" s="3">
         <v>48.377823392231399</v>
       </c>
-      <c r="L8" s="4">
+      <c r="L8" s="3">
         <v>72.790878504914801</v>
       </c>
-      <c r="M8" s="4">
+      <c r="M8" s="3">
         <v>150.069685656758</v>
       </c>
-      <c r="N8" s="4">
+      <c r="N8" s="3">
         <v>227.34818345797899</v>
       </c>
-      <c r="O8" s="4">
+      <c r="O8" s="3">
         <v>304.626897404499</v>
       </c>
-      <c r="P8" s="4">
+      <c r="P8" s="3">
         <v>381.90539520572003</v>
       </c>
-      <c r="Q8" s="4">
+      <c r="Q8" s="3">
         <v>459.18370196002297</v>
       </c>
-      <c r="R8" s="4">
+      <c r="R8" s="3">
         <v>536.46181083334204</v>
       </c>
-      <c r="S8" s="4">
+      <c r="S8" s="3">
         <v>702.82497272727301</v>
       </c>
-      <c r="T8" s="4">
+      <c r="T8" s="3">
         <v>868.19555454545502</v>
       </c>
-      <c r="U8" s="4">
+      <c r="U8" s="3">
         <v>1033.56613636364</v>
       </c>
-      <c r="V8" s="4">
+      <c r="V8" s="3">
         <v>1198.93671818182</v>
       </c>
-      <c r="W8" s="4">
+      <c r="W8" s="3">
         <v>1343.6359772727301</v>
       </c>
-      <c r="X8" s="4">
+      <c r="X8" s="3">
         <v>1467.6639136363599</v>
       </c>
-      <c r="Y8" s="4">
+      <c r="Y8" s="3">
         <v>1529.6778818181799</v>
       </c>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="H9" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="I9" s="4">
-        <v>0</v>
-      </c>
-      <c r="J9" s="4">
+      <c r="I9" s="3">
+        <v>0</v>
+      </c>
+      <c r="J9" s="3">
         <v>0.53980634214760304</v>
       </c>
-      <c r="K9" s="4">
+      <c r="K9" s="3">
         <v>0.84225168111512305</v>
       </c>
-      <c r="L9" s="4">
+      <c r="L9" s="3">
         <v>0.81562484681338399</v>
       </c>
-      <c r="M9" s="4">
+      <c r="M9" s="3">
         <v>0.73415517130997998</v>
       </c>
-      <c r="N9" s="4">
+      <c r="N9" s="3">
         <v>101.112293090967</v>
       </c>
-      <c r="O9" s="4">
+      <c r="O9" s="3">
         <v>291.14253494945598</v>
       </c>
-      <c r="P9" s="4"/>
-      <c r="Q9" s="4">
+      <c r="P9" s="3"/>
+      <c r="Q9" s="3">
         <v>988.70810483387697</v>
       </c>
-      <c r="R9" s="4"/>
-      <c r="S9" s="4">
+      <c r="R9" s="3"/>
+      <c r="S9" s="3">
         <v>1189.9939971654401</v>
       </c>
-      <c r="T9" s="4"/>
-      <c r="U9" s="4">
+      <c r="T9" s="3"/>
+      <c r="U9" s="3">
         <v>1204.9152962651799</v>
       </c>
-      <c r="V9" s="4"/>
-      <c r="W9" s="4">
+      <c r="V9" s="3"/>
+      <c r="W9" s="3">
         <v>1207.7756876621299</v>
       </c>
-      <c r="X9" s="4"/>
-      <c r="Y9" s="4">
+      <c r="X9" s="3"/>
+      <c r="Y9" s="3">
         <v>1208.3173630809999</v>
       </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="H10" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="I10" s="4">
-        <v>0</v>
-      </c>
-      <c r="J10" s="4">
-        <v>0</v>
-      </c>
-      <c r="K10" s="4">
+      <c r="I10" s="3">
+        <v>0</v>
+      </c>
+      <c r="J10" s="3">
+        <v>0</v>
+      </c>
+      <c r="K10" s="3">
         <v>266.7382533</v>
       </c>
-      <c r="L10" s="4">
+      <c r="L10" s="3">
         <v>266.7382533</v>
       </c>
-      <c r="M10" s="4">
+      <c r="M10" s="3">
         <v>65.804774046930504</v>
       </c>
-      <c r="N10" s="4">
+      <c r="N10" s="3">
         <v>83.985419840575901</v>
       </c>
-      <c r="O10" s="4">
+      <c r="O10" s="3">
         <v>107.18904286134899</v>
       </c>
-      <c r="P10" s="4">
+      <c r="P10" s="3">
         <v>136.803399105962</v>
       </c>
-      <c r="Q10" s="4">
+      <c r="Q10" s="3">
         <v>174.59965596626799</v>
       </c>
-      <c r="R10" s="4"/>
-      <c r="S10" s="4">
+      <c r="R10" s="3"/>
+      <c r="S10" s="3">
         <v>249.88511625801499</v>
       </c>
-      <c r="T10" s="4"/>
-      <c r="U10" s="4">
+      <c r="T10" s="3"/>
+      <c r="U10" s="3">
         <v>407.03652318433598</v>
       </c>
-      <c r="V10" s="4"/>
-      <c r="W10" s="4">
+      <c r="V10" s="3"/>
+      <c r="W10" s="3">
         <v>663.01960551713796</v>
       </c>
-      <c r="X10" s="4"/>
-      <c r="Y10" s="4">
+      <c r="X10" s="3"/>
+      <c r="Y10" s="3">
         <v>1079.9890728749599</v>
       </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="H11" s="4" t="s">
+      <c r="H11" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="I11" s="4">
+      <c r="I11" s="3">
         <v>11.893366739519999</v>
       </c>
-      <c r="J11" s="4">
+      <c r="J11" s="3">
         <v>14.778382171200001</v>
       </c>
-      <c r="K11" s="4">
+      <c r="K11" s="3">
         <v>22.103587080960001</v>
       </c>
-      <c r="L11" s="4">
+      <c r="L11" s="3">
         <v>34.410645812879999</v>
       </c>
-      <c r="M11" s="4">
+      <c r="M11" s="3">
         <v>47.942128747680002</v>
       </c>
-      <c r="N11" s="4">
+      <c r="N11" s="3">
         <v>66.6504870192</v>
       </c>
-      <c r="O11" s="4">
+      <c r="O11" s="3">
         <v>93.178825847040002</v>
       </c>
-      <c r="P11" s="4">
+      <c r="P11" s="3">
         <v>129.73780941935999</v>
       </c>
-      <c r="Q11" s="4">
+      <c r="Q11" s="3">
         <v>180.11050925232001</v>
       </c>
-      <c r="R11" s="4"/>
-      <c r="S11" s="4">
+      <c r="R11" s="3"/>
+      <c r="S11" s="3">
         <v>315.72246535272001</v>
       </c>
-      <c r="T11" s="4"/>
-      <c r="U11" s="4">
+      <c r="T11" s="3"/>
+      <c r="U11" s="3">
         <v>490.30733443295998</v>
       </c>
-      <c r="V11" s="4"/>
-      <c r="W11" s="4">
+      <c r="V11" s="3"/>
+      <c r="W11" s="3">
         <v>761.43229761696</v>
       </c>
-      <c r="X11" s="4"/>
-      <c r="Y11" s="4">
+      <c r="X11" s="3"/>
+      <c r="Y11" s="3">
         <v>1182.48107496528</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="H12" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="I12" s="4">
+      <c r="I12" s="3">
         <v>1.0990177343346599E-12</v>
       </c>
-      <c r="J12" s="4">
+      <c r="J12" s="3">
         <v>5.2952864058353004</v>
       </c>
-      <c r="K12" s="4">
+      <c r="K12" s="3">
         <v>5.2078813347109003</v>
       </c>
-      <c r="L12" s="4">
+      <c r="L12" s="3">
         <v>26.8664890015453</v>
       </c>
-      <c r="M12" s="4">
+      <c r="M12" s="3">
         <v>30.507434024116598</v>
       </c>
-      <c r="N12" s="4">
+      <c r="N12" s="3">
         <v>69.7228875107444</v>
       </c>
-      <c r="O12" s="4">
+      <c r="O12" s="3">
         <v>161.962406279503</v>
       </c>
-      <c r="P12" s="4">
+      <c r="P12" s="3">
         <v>315.37978828260998</v>
       </c>
-      <c r="Q12" s="4">
+      <c r="Q12" s="3">
         <v>425.64693327013703</v>
       </c>
-      <c r="R12" s="4">
+      <c r="R12" s="3">
         <v>575.73546541505698</v>
       </c>
-      <c r="S12" s="4">
+      <c r="S12" s="3">
         <v>652.972841797466</v>
       </c>
-      <c r="T12" s="4">
+      <c r="T12" s="3">
         <v>742.228583268482</v>
       </c>
-      <c r="U12" s="4">
+      <c r="U12" s="3">
         <v>831.86132623401704</v>
       </c>
-      <c r="V12" s="4">
+      <c r="V12" s="3">
         <v>921.51531852568701</v>
       </c>
-      <c r="W12" s="4">
+      <c r="W12" s="3">
         <v>1011.16942729356</v>
       </c>
-      <c r="X12" s="4">
+      <c r="X12" s="3">
         <v>1100.8222245202701</v>
       </c>
-      <c r="Y12" s="4">
+      <c r="Y12" s="3">
         <v>1190.4744313116</v>
       </c>
     </row>
@@ -1906,80 +2000,80 @@
         <v>3.9050687686204499</v>
       </c>
     </row>
-    <row r="18" spans="1:25" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="6" t="s">
+    <row r="18" spans="1:25" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E18" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="F18" s="6" t="s">
+      <c r="E18" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="F18" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="G18" s="6" t="s">
+      <c r="G18" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="H18" s="6" t="s">
+      <c r="H18" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="I18" s="6">
+      <c r="I18" s="5">
         <v>4.2937118560110198E-6</v>
       </c>
-      <c r="J18" s="6">
+      <c r="J18" s="5">
         <v>-4.2292770401243102E-2</v>
       </c>
-      <c r="K18" s="6">
+      <c r="K18" s="5">
         <v>0.222225947812831</v>
       </c>
-      <c r="L18" s="6">
+      <c r="L18" s="5">
         <v>1.7126069263166299</v>
       </c>
-      <c r="M18" s="6">
+      <c r="M18" s="5">
         <v>4.0494873993390303</v>
       </c>
-      <c r="N18" s="6">
+      <c r="N18" s="5">
         <v>6.5525850910371002</v>
       </c>
-      <c r="O18" s="6">
+      <c r="O18" s="5">
         <v>8.3118774968184095</v>
       </c>
-      <c r="P18" s="6">
+      <c r="P18" s="5">
         <v>9.3987358937538907</v>
       </c>
-      <c r="Q18" s="6">
+      <c r="Q18" s="5">
         <v>10.0159828085178</v>
       </c>
-      <c r="R18" s="6">
+      <c r="R18" s="5">
         <v>10.2903428613829</v>
       </c>
-      <c r="S18" s="6">
+      <c r="S18" s="5">
         <v>10.210168333908801</v>
       </c>
-      <c r="T18" s="6">
+      <c r="T18" s="5">
         <v>9.7292197199435009</v>
       </c>
-      <c r="U18" s="6">
+      <c r="U18" s="5">
         <v>8.9547284462648093</v>
       </c>
-      <c r="V18" s="6">
+      <c r="V18" s="5">
         <v>7.8111494616878296</v>
       </c>
-      <c r="W18" s="6">
+      <c r="W18" s="5">
         <v>6.3003742918332897</v>
       </c>
-      <c r="X18" s="6">
+      <c r="X18" s="5">
         <v>4.4075455817190496</v>
       </c>
-      <c r="Y18" s="6">
+      <c r="Y18" s="5">
         <v>2.1330977064349899</v>
       </c>
     </row>
@@ -2368,77 +2462,77 @@
         <v>-29.054093676522498</v>
       </c>
     </row>
-    <row r="24" spans="1:25" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="6" t="s">
+    <row r="24" spans="1:25" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="D24" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E24" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="F24" s="6" t="s">
+      <c r="E24" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="F24" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="G24" s="6" t="s">
+      <c r="G24" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="H24" s="6" t="s">
+      <c r="H24" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="I24" s="6">
+      <c r="I24" s="5">
         <v>-1.05356954453554E-3</v>
       </c>
-      <c r="J24" s="6">
+      <c r="J24" s="5">
         <v>-6.1256134953197798E-4</v>
       </c>
-      <c r="K24" s="6">
+      <c r="K24" s="5">
         <v>5.8999414468719799E-2</v>
       </c>
-      <c r="L24" s="6">
+      <c r="L24" s="5">
         <v>0.53222945241509201</v>
       </c>
-      <c r="M24" s="6">
+      <c r="M24" s="5">
         <v>1.8371641778094401</v>
       </c>
-      <c r="N24" s="6">
+      <c r="N24" s="5">
         <v>3.3676635324655302</v>
       </c>
       <c r="O24" s="1">
         <v>4.1759243551226204</v>
       </c>
-      <c r="P24" s="6">
+      <c r="P24" s="5">
         <v>3.5239742153448401</v>
       </c>
-      <c r="Q24" s="6">
+      <c r="Q24" s="5">
         <v>4.6076488949428898</v>
       </c>
-      <c r="R24" s="6">
+      <c r="R24" s="5">
         <v>7.0595305652515901</v>
       </c>
-      <c r="S24" s="6">
+      <c r="S24" s="5">
         <v>6.7984408470273499</v>
       </c>
-      <c r="T24" s="6">
+      <c r="T24" s="5">
         <v>6.2792827798665396</v>
       </c>
-      <c r="U24" s="6">
+      <c r="U24" s="5">
         <v>5.5871110190111404</v>
       </c>
-      <c r="V24" s="6">
+      <c r="V24" s="5">
         <v>4.61855048253652</v>
       </c>
-      <c r="W24" s="6">
+      <c r="W24" s="5">
         <v>3.1346955366020399</v>
       </c>
-      <c r="X24" s="6">
+      <c r="X24" s="5">
         <v>0.94331950537928599</v>
       </c>
       <c r="Y24" s="1">
@@ -2830,80 +2924,80 @@
         <v>-30.924750737664699</v>
       </c>
     </row>
-    <row r="30" spans="1:25" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="8" t="s">
+    <row r="30" spans="1:25" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C30" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D30" s="9" t="s">
+      <c r="D30" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="E30" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="F30" s="9" t="s">
+      <c r="E30" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="F30" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="G30" s="9" t="s">
+      <c r="G30" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="H30" s="9" t="s">
+      <c r="H30" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="I30" s="9">
+      <c r="I30" s="8">
         <v>-8.7913750073166999E-4</v>
       </c>
-      <c r="J30" s="9">
+      <c r="J30" s="8">
         <v>-5.8332650511705799E-4</v>
       </c>
-      <c r="K30" s="9">
+      <c r="K30" s="8">
         <v>-0.36260718770109401</v>
       </c>
-      <c r="L30" s="9">
+      <c r="L30" s="8">
         <v>-0.70973931104547405</v>
       </c>
-      <c r="M30" s="9">
+      <c r="M30" s="8">
         <v>-0.46387274310988502</v>
       </c>
-      <c r="N30" s="9">
+      <c r="N30" s="8">
         <v>-1.0911267095544599</v>
       </c>
-      <c r="O30" s="10">
+      <c r="O30" s="9">
         <v>-1.6434290536272</v>
       </c>
-      <c r="P30" s="9">
+      <c r="P30" s="8">
         <v>-2.4881449937226998</v>
       </c>
-      <c r="Q30" s="9">
+      <c r="Q30" s="8">
         <v>-3.1756219186050401</v>
       </c>
-      <c r="R30" s="9">
+      <c r="R30" s="8">
         <v>-3.7951404595943199</v>
       </c>
-      <c r="S30" s="9">
+      <c r="S30" s="8">
         <v>-4.9206087414089499</v>
       </c>
-      <c r="T30" s="11">
+      <c r="T30" s="10">
         <v>-5.3157227290386002</v>
       </c>
-      <c r="U30" s="9">
+      <c r="U30" s="8">
         <v>-4.0423714719693598</v>
       </c>
-      <c r="V30" s="9">
+      <c r="V30" s="8">
         <v>-5.2003308370125598</v>
       </c>
-      <c r="W30" s="9">
+      <c r="W30" s="8">
         <v>-4.7058093442706799</v>
       </c>
-      <c r="X30" s="9">
+      <c r="X30" s="8">
         <v>-4.3698814438566904</v>
       </c>
-      <c r="Y30" s="10">
+      <c r="Y30" s="9">
         <v>-3.7840036088050302</v>
       </c>
     </row>
@@ -3292,7 +3386,7 @@
         <v>-28.7761901081358</v>
       </c>
     </row>
-    <row r="36" spans="1:25" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:25" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>25</v>
       </c>
@@ -3754,80 +3848,80 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:25" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="6" t="s">
+    <row r="42" spans="1:25" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="B42" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C42" s="6" t="s">
+      <c r="C42" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D42" s="6" t="s">
+      <c r="D42" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E42" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="F42" s="6" t="s">
+      <c r="E42" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="F42" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G42" s="6" t="s">
+      <c r="G42" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="H42" s="6" t="s">
+      <c r="H42" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="I42" s="6">
-        <v>0</v>
-      </c>
-      <c r="J42" s="6">
-        <v>0</v>
-      </c>
-      <c r="K42" s="6">
-        <v>0</v>
-      </c>
-      <c r="L42" s="6">
-        <v>0</v>
-      </c>
-      <c r="M42" s="6">
-        <v>0</v>
-      </c>
-      <c r="N42" s="6">
-        <v>0</v>
-      </c>
-      <c r="O42" s="6">
-        <v>0</v>
-      </c>
-      <c r="P42" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q42" s="6">
-        <v>0</v>
-      </c>
-      <c r="R42" s="6">
-        <v>0</v>
-      </c>
-      <c r="S42" s="6">
-        <v>0</v>
-      </c>
-      <c r="T42" s="6">
-        <v>0</v>
-      </c>
-      <c r="U42" s="6">
-        <v>0</v>
-      </c>
-      <c r="V42" s="6">
-        <v>0</v>
-      </c>
-      <c r="W42" s="6">
-        <v>0</v>
-      </c>
-      <c r="X42" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y42" s="6">
+      <c r="I42" s="5">
+        <v>0</v>
+      </c>
+      <c r="J42" s="5">
+        <v>0</v>
+      </c>
+      <c r="K42" s="5">
+        <v>0</v>
+      </c>
+      <c r="L42" s="5">
+        <v>0</v>
+      </c>
+      <c r="M42" s="5">
+        <v>0</v>
+      </c>
+      <c r="N42" s="5">
+        <v>0</v>
+      </c>
+      <c r="O42" s="5">
+        <v>0</v>
+      </c>
+      <c r="P42" s="5">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="5">
+        <v>0</v>
+      </c>
+      <c r="R42" s="5">
+        <v>0</v>
+      </c>
+      <c r="S42" s="5">
+        <v>0</v>
+      </c>
+      <c r="T42" s="5">
+        <v>0</v>
+      </c>
+      <c r="U42" s="5">
+        <v>0</v>
+      </c>
+      <c r="V42" s="5">
+        <v>0</v>
+      </c>
+      <c r="W42" s="5">
+        <v>0</v>
+      </c>
+      <c r="X42" s="5">
+        <v>0</v>
+      </c>
+      <c r="Y42" s="5">
         <v>0</v>
       </c>
     </row>
@@ -4216,80 +4310,80 @@
         <v>-21.6587757424378</v>
       </c>
     </row>
-    <row r="48" spans="1:25" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="6" t="s">
+    <row r="48" spans="1:25" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B48" s="6" t="s">
+      <c r="B48" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C48" s="6" t="s">
+      <c r="C48" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D48" s="6" t="s">
+      <c r="D48" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E48" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="F48" s="6" t="s">
+      <c r="E48" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="F48" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G48" s="6" t="s">
+      <c r="G48" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="H48" s="6" t="s">
+      <c r="H48" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="I48" s="6">
+      <c r="I48" s="5">
         <v>-4.8116408388063601E-4</v>
       </c>
-      <c r="J48" s="6">
+      <c r="J48" s="5">
         <v>6.5778399950188805E-5</v>
       </c>
-      <c r="K48" s="6">
+      <c r="K48" s="5">
         <v>4.4460659212569198E-2</v>
       </c>
-      <c r="L48" s="6">
+      <c r="L48" s="5">
         <v>2.2152483096230598E-3</v>
       </c>
-      <c r="M48" s="6">
+      <c r="M48" s="5">
         <v>-2.6005910209274299E-2</v>
       </c>
-      <c r="N48" s="6">
+      <c r="N48" s="5">
         <v>-3.2841559460654299E-2</v>
       </c>
-      <c r="O48" s="6">
+      <c r="O48" s="5">
         <v>-5.7055621910321798E-2</v>
       </c>
-      <c r="P48" s="6">
+      <c r="P48" s="5">
         <v>-4.3408051781953901E-2</v>
       </c>
-      <c r="Q48" s="6">
+      <c r="Q48" s="5">
         <v>-0.354280079858458</v>
       </c>
-      <c r="R48" s="6">
+      <c r="R48" s="5">
         <v>-1.0129346962212</v>
       </c>
-      <c r="S48" s="6">
+      <c r="S48" s="5">
         <v>-1.6859498767372101</v>
       </c>
-      <c r="T48" s="6">
+      <c r="T48" s="5">
         <v>-2.3255091075405199</v>
       </c>
-      <c r="U48" s="6">
+      <c r="U48" s="5">
         <v>-3.15034260913029</v>
       </c>
-      <c r="V48" s="6">
+      <c r="V48" s="5">
         <v>-3.9500565454043302</v>
       </c>
-      <c r="W48" s="6">
+      <c r="W48" s="5">
         <v>-3.9622315664754701</v>
       </c>
-      <c r="X48" s="6">
+      <c r="X48" s="5">
         <v>-3.01483067186612</v>
       </c>
-      <c r="Y48" s="6">
+      <c r="Y48" s="5">
         <v>-3.3281006635520902</v>
       </c>
     </row>
@@ -4678,80 +4772,80 @@
         <v>-43.204864542108602</v>
       </c>
     </row>
-    <row r="54" spans="1:25" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="8" t="s">
+    <row r="54" spans="1:25" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B54" s="9" t="s">
+      <c r="B54" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C54" s="9" t="s">
+      <c r="C54" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D54" s="9" t="s">
+      <c r="D54" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="E54" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="F54" s="9" t="s">
+      <c r="E54" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="F54" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="G54" s="9" t="s">
+      <c r="G54" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="H54" s="9" t="s">
+      <c r="H54" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="I54" s="9">
+      <c r="I54" s="8">
         <v>-6.4526438354928402E-4</v>
       </c>
-      <c r="J54" s="9">
+      <c r="J54" s="8">
         <v>-2.8138537756838898E-4</v>
       </c>
-      <c r="K54" s="9">
+      <c r="K54" s="8">
         <v>-0.18662432866873499</v>
       </c>
-      <c r="L54" s="9">
+      <c r="L54" s="8">
         <v>-2.2820558133245901</v>
       </c>
-      <c r="M54" s="9">
+      <c r="M54" s="8">
         <v>-2.0152449032145299</v>
       </c>
-      <c r="N54" s="9">
+      <c r="N54" s="8">
         <v>-2.9417147205340601</v>
       </c>
-      <c r="O54" s="10">
+      <c r="O54" s="9">
         <v>-3.5465996387186798</v>
       </c>
-      <c r="P54" s="9">
+      <c r="P54" s="8">
         <v>-4.8331370562782396</v>
       </c>
-      <c r="Q54" s="11">
+      <c r="Q54" s="10">
         <v>-6.4120026541508004</v>
       </c>
-      <c r="R54" s="9">
+      <c r="R54" s="8">
         <v>-5.8685094717820796</v>
       </c>
-      <c r="S54" s="9">
+      <c r="S54" s="8">
         <v>-4.97600469012826</v>
       </c>
-      <c r="T54" s="9">
+      <c r="T54" s="8">
         <v>-5.1867705410924403</v>
       </c>
-      <c r="U54" s="9">
+      <c r="U54" s="8">
         <v>-5.1431987307323697</v>
       </c>
-      <c r="V54" s="9">
+      <c r="V54" s="8">
         <v>-5.1449302502717504</v>
       </c>
-      <c r="W54" s="9">
+      <c r="W54" s="8">
         <v>-5.1915414749731097</v>
       </c>
-      <c r="X54" s="9">
+      <c r="X54" s="8">
         <v>-5.2318674913929</v>
       </c>
-      <c r="Y54" s="10">
+      <c r="Y54" s="9">
         <v>-5.14824197838725</v>
       </c>
     </row>
@@ -5140,80 +5234,80 @@
         <v>-42.033242124051199</v>
       </c>
     </row>
-    <row r="60" spans="1:25" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="6" t="s">
+    <row r="60" spans="1:25" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A60" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B60" s="6" t="s">
+      <c r="B60" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C60" s="6" t="s">
+      <c r="C60" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D60" s="6" t="s">
+      <c r="D60" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E60" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="F60" s="6" t="s">
+      <c r="E60" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="F60" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="G60" s="6" t="s">
+      <c r="G60" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="H60" s="6" t="s">
+      <c r="H60" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="I60" s="6">
+      <c r="I60" s="5">
         <v>-7.5139957187309796E-6</v>
       </c>
-      <c r="J60" s="6">
+      <c r="J60" s="5">
         <v>-4.2332854113705499E-2</v>
       </c>
-      <c r="K60" s="6">
+      <c r="K60" s="5">
         <v>-0.251566784356899</v>
       </c>
-      <c r="L60" s="6">
+      <c r="L60" s="5">
         <v>-2.1612216017999</v>
       </c>
-      <c r="M60" s="6">
+      <c r="M60" s="5">
         <v>-5.2706006448886296</v>
       </c>
-      <c r="N60" s="6">
+      <c r="N60" s="5">
         <v>-9.0451643508747992</v>
       </c>
-      <c r="O60" s="6">
+      <c r="O60" s="5">
         <v>-12.8399892026162</v>
       </c>
-      <c r="P60" s="6">
+      <c r="P60" s="5">
         <v>-16.453941433097501</v>
       </c>
-      <c r="Q60" s="6">
+      <c r="Q60" s="5">
         <v>-20.013063727353501</v>
       </c>
-      <c r="R60" s="6">
+      <c r="R60" s="5">
         <v>-23.474302237939298</v>
       </c>
-      <c r="S60" s="6">
+      <c r="S60" s="5">
         <v>-26.753629415896</v>
       </c>
-      <c r="T60" s="6">
+      <c r="T60" s="5">
         <v>-29.809657846262599</v>
       </c>
-      <c r="U60" s="6">
+      <c r="U60" s="5">
         <v>-32.544644220651101</v>
       </c>
-      <c r="V60" s="6">
+      <c r="V60" s="5">
         <v>-34.972324537001398</v>
       </c>
-      <c r="W60" s="6">
+      <c r="W60" s="5">
         <v>-37.116166261611603</v>
       </c>
-      <c r="X60" s="6">
+      <c r="X60" s="5">
         <v>-39.047093763077001</v>
       </c>
-      <c r="Y60" s="6">
+      <c r="Y60" s="5">
         <v>-40.7958520961541</v>
       </c>
     </row>
@@ -5602,80 +5696,80 @@
         <v>76.393144966072995</v>
       </c>
     </row>
-    <row r="66" spans="1:25" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="6" t="s">
+    <row r="66" spans="1:25" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A66" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B66" s="6" t="s">
+      <c r="B66" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C66" s="6" t="s">
+      <c r="C66" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D66" s="6" t="s">
+      <c r="D66" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E66" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="F66" s="6" t="s">
+      <c r="E66" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="F66" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="G66" s="6" t="s">
+      <c r="G66" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="H66" s="6" t="s">
+      <c r="H66" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="I66" s="6">
+      <c r="I66" s="5">
         <v>7.1114602529758301E-6</v>
       </c>
-      <c r="J66" s="6">
+      <c r="J66" s="5">
         <v>-4.2295054373455702E-2</v>
       </c>
-      <c r="K66" s="6">
+      <c r="K66" s="5">
         <v>0.48317339515674002</v>
       </c>
-      <c r="L66" s="6">
+      <c r="L66" s="5">
         <v>4.22939452747503</v>
       </c>
-      <c r="M66" s="6">
+      <c r="M66" s="5">
         <v>10.7650882437483</v>
       </c>
-      <c r="N66" s="6">
+      <c r="N66" s="5">
         <v>18.331249328206699</v>
       </c>
-      <c r="O66" s="6">
+      <c r="O66" s="5">
         <v>24.996178231193099</v>
       </c>
-      <c r="P66" s="6">
+      <c r="P66" s="5">
         <v>30.9749987744595</v>
       </c>
-      <c r="Q66" s="6">
+      <c r="Q66" s="5">
         <v>36.656762176677397</v>
       </c>
-      <c r="R66" s="6">
+      <c r="R66" s="5">
         <v>42.167141441038602</v>
       </c>
-      <c r="S66" s="6">
+      <c r="S66" s="5">
         <v>47.426640369723103</v>
       </c>
-      <c r="T66" s="6">
+      <c r="T66" s="5">
         <v>52.2865281663899</v>
       </c>
-      <c r="U66" s="6">
+      <c r="U66" s="5">
         <v>56.841740059922301</v>
       </c>
-      <c r="V66" s="6">
+      <c r="V66" s="5">
         <v>60.937839357793003</v>
       </c>
-      <c r="W66" s="6">
+      <c r="W66" s="5">
         <v>64.509733111129606</v>
       </c>
-      <c r="X66" s="6">
+      <c r="X66" s="5">
         <v>67.441465769056506</v>
       </c>
-      <c r="Y66" s="6">
+      <c r="Y66" s="5">
         <v>69.640017031649293</v>
       </c>
     </row>
@@ -6064,80 +6158,80 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:25" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="7" t="s">
+    <row r="72" spans="1:25" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A72" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="B72" s="7" t="s">
+      <c r="B72" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C72" s="7" t="s">
+      <c r="C72" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D72" s="7" t="s">
+      <c r="D72" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="E72" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="F72" s="7" t="s">
+      <c r="E72" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F72" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="G72" s="7" t="s">
+      <c r="G72" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="H72" s="7" t="s">
+      <c r="H72" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="I72" s="7">
-        <v>0</v>
-      </c>
-      <c r="J72" s="7">
-        <v>0</v>
-      </c>
-      <c r="K72" s="7">
-        <v>0</v>
-      </c>
-      <c r="L72" s="7">
-        <v>0</v>
-      </c>
-      <c r="M72" s="7">
-        <v>0</v>
-      </c>
-      <c r="N72" s="7">
-        <v>0</v>
-      </c>
-      <c r="O72" s="7">
-        <v>0</v>
-      </c>
-      <c r="P72" s="7">
-        <v>0</v>
-      </c>
-      <c r="Q72" s="7">
-        <v>0</v>
-      </c>
-      <c r="R72" s="7">
-        <v>0</v>
-      </c>
-      <c r="S72" s="7">
-        <v>0</v>
-      </c>
-      <c r="T72" s="7">
-        <v>0</v>
-      </c>
-      <c r="U72" s="7">
-        <v>0</v>
-      </c>
-      <c r="V72" s="7">
-        <v>0</v>
-      </c>
-      <c r="W72" s="7">
-        <v>0</v>
-      </c>
-      <c r="X72" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y72" s="7">
+      <c r="I72" s="6">
+        <v>0</v>
+      </c>
+      <c r="J72" s="6">
+        <v>0</v>
+      </c>
+      <c r="K72" s="6">
+        <v>0</v>
+      </c>
+      <c r="L72" s="6">
+        <v>0</v>
+      </c>
+      <c r="M72" s="6">
+        <v>0</v>
+      </c>
+      <c r="N72" s="6">
+        <v>0</v>
+      </c>
+      <c r="O72" s="6">
+        <v>0</v>
+      </c>
+      <c r="P72" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q72" s="6">
+        <v>0</v>
+      </c>
+      <c r="R72" s="6">
+        <v>0</v>
+      </c>
+      <c r="S72" s="6">
+        <v>0</v>
+      </c>
+      <c r="T72" s="6">
+        <v>0</v>
+      </c>
+      <c r="U72" s="6">
+        <v>0</v>
+      </c>
+      <c r="V72" s="6">
+        <v>0</v>
+      </c>
+      <c r="W72" s="6">
+        <v>0</v>
+      </c>
+      <c r="X72" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y72" s="6">
         <v>0</v>
       </c>
     </row>
@@ -6451,70 +6545,70 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:25" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="7" t="s">
+    <row r="78" spans="1:25" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A78" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B78" s="7" t="s">
+      <c r="B78" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C78" s="7" t="s">
+      <c r="C78" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D78" s="7" t="s">
+      <c r="D78" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="E78" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="F78" s="7" t="s">
+      <c r="E78" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F78" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="G78" s="7" t="s">
+      <c r="G78" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="H78" s="7" t="s">
+      <c r="H78" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I78" s="7">
-        <v>0</v>
-      </c>
-      <c r="J78" s="7">
-        <v>0</v>
-      </c>
-      <c r="K78" s="7">
-        <v>0</v>
-      </c>
-      <c r="L78" s="7">
-        <v>0</v>
-      </c>
-      <c r="M78" s="7">
-        <v>0</v>
-      </c>
-      <c r="N78" s="7">
-        <v>0</v>
-      </c>
-      <c r="O78" s="7">
-        <v>0</v>
-      </c>
-      <c r="P78" s="7"/>
-      <c r="Q78" s="7">
-        <v>0</v>
-      </c>
-      <c r="R78" s="7"/>
-      <c r="S78" s="7">
-        <v>0</v>
-      </c>
-      <c r="T78" s="7"/>
-      <c r="U78" s="7">
-        <v>0</v>
-      </c>
-      <c r="V78" s="7"/>
-      <c r="W78" s="7">
-        <v>0</v>
-      </c>
-      <c r="X78" s="7"/>
-      <c r="Y78" s="7">
+      <c r="I78" s="6">
+        <v>0</v>
+      </c>
+      <c r="J78" s="6">
+        <v>0</v>
+      </c>
+      <c r="K78" s="6">
+        <v>0</v>
+      </c>
+      <c r="L78" s="6">
+        <v>0</v>
+      </c>
+      <c r="M78" s="6">
+        <v>0</v>
+      </c>
+      <c r="N78" s="6">
+        <v>0</v>
+      </c>
+      <c r="O78" s="6">
+        <v>0</v>
+      </c>
+      <c r="P78" s="6"/>
+      <c r="Q78" s="6">
+        <v>0</v>
+      </c>
+      <c r="R78" s="6"/>
+      <c r="S78" s="6">
+        <v>0</v>
+      </c>
+      <c r="T78" s="6"/>
+      <c r="U78" s="6">
+        <v>0</v>
+      </c>
+      <c r="V78" s="6"/>
+      <c r="W78" s="6">
+        <v>0</v>
+      </c>
+      <c r="X78" s="6"/>
+      <c r="Y78" s="6">
         <v>0</v>
       </c>
     </row>
@@ -6843,72 +6937,72 @@
         <v>-2.6942045543046498</v>
       </c>
     </row>
-    <row r="84" spans="1:25" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A84" s="7" t="s">
+    <row r="84" spans="1:25" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A84" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B84" s="7" t="s">
+      <c r="B84" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C84" s="7" t="s">
+      <c r="C84" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D84" s="7" t="s">
+      <c r="D84" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="E84" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="F84" s="7" t="s">
+      <c r="E84" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F84" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="G84" s="7" t="s">
+      <c r="G84" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="H84" s="7" t="s">
+      <c r="H84" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="I84" s="7">
-        <v>0</v>
-      </c>
-      <c r="J84" s="7">
-        <v>0</v>
-      </c>
-      <c r="K84" s="7">
-        <v>0</v>
-      </c>
-      <c r="L84" s="7">
-        <v>0</v>
-      </c>
-      <c r="M84" s="7">
+      <c r="I84" s="6">
+        <v>0</v>
+      </c>
+      <c r="J84" s="6">
+        <v>0</v>
+      </c>
+      <c r="K84" s="6">
+        <v>0</v>
+      </c>
+      <c r="L84" s="6">
+        <v>0</v>
+      </c>
+      <c r="M84" s="6">
         <v>-0.25683724755368498</v>
       </c>
-      <c r="N84" s="7">
+      <c r="N84" s="6">
         <v>-0.40178370708142302</v>
       </c>
-      <c r="O84" s="7">
+      <c r="O84" s="6">
         <v>-0.50515465460651199</v>
       </c>
-      <c r="P84" s="7">
+      <c r="P84" s="6">
         <v>-0.56171201737101795</v>
       </c>
-      <c r="Q84" s="7">
+      <c r="Q84" s="6">
         <v>-0.58916408754758898</v>
       </c>
-      <c r="R84" s="7"/>
-      <c r="S84" s="7">
+      <c r="R84" s="6"/>
+      <c r="S84" s="6">
         <v>-0.59605323085745299</v>
       </c>
-      <c r="T84" s="7"/>
-      <c r="U84" s="7">
+      <c r="T84" s="6"/>
+      <c r="U84" s="6">
         <v>-0.65033728169680305</v>
       </c>
-      <c r="V84" s="7"/>
-      <c r="W84" s="7">
+      <c r="V84" s="6"/>
+      <c r="W84" s="6">
         <v>-0.67455974529174201</v>
       </c>
-      <c r="X84" s="7"/>
-      <c r="Y84" s="7">
+      <c r="X84" s="6"/>
+      <c r="Y84" s="6">
         <v>-0.723350261433785</v>
       </c>
     </row>
@@ -7237,72 +7331,72 @@
         <v>1.39337017704445</v>
       </c>
     </row>
-    <row r="90" spans="1:25" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A90" s="7" t="s">
+    <row r="90" spans="1:25" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A90" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B90" s="7" t="s">
+      <c r="B90" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C90" s="7" t="s">
+      <c r="C90" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D90" s="7" t="s">
+      <c r="D90" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="E90" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="F90" s="7" t="s">
+      <c r="E90" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F90" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="G90" s="7" t="s">
+      <c r="G90" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="H90" s="7" t="s">
+      <c r="H90" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="I90" s="7">
-        <v>0</v>
-      </c>
-      <c r="J90" s="7">
-        <v>0</v>
-      </c>
-      <c r="K90" s="7">
-        <v>0</v>
-      </c>
-      <c r="L90" s="7">
+      <c r="I90" s="6">
+        <v>0</v>
+      </c>
+      <c r="J90" s="6">
+        <v>0</v>
+      </c>
+      <c r="K90" s="6">
+        <v>0</v>
+      </c>
+      <c r="L90" s="6">
         <v>2.2815597383173E-2</v>
       </c>
-      <c r="M90" s="7">
+      <c r="M90" s="6">
         <v>-9.4524263376581596E-2</v>
       </c>
-      <c r="N90" s="7">
+      <c r="N90" s="6">
         <v>-0.19136244074762601</v>
       </c>
-      <c r="O90" s="7">
+      <c r="O90" s="6">
         <v>-0.36694415702604899</v>
       </c>
-      <c r="P90" s="7">
+      <c r="P90" s="6">
         <v>-0.57071685011872697</v>
       </c>
-      <c r="Q90" s="7">
+      <c r="Q90" s="6">
         <v>-0.733153960792848</v>
       </c>
-      <c r="R90" s="7"/>
-      <c r="S90" s="7">
+      <c r="R90" s="6"/>
+      <c r="S90" s="6">
         <v>-1.1597849085932499</v>
       </c>
-      <c r="T90" s="7"/>
-      <c r="U90" s="7">
+      <c r="T90" s="6"/>
+      <c r="U90" s="6">
         <v>-1.4235285366596699</v>
       </c>
-      <c r="V90" s="7"/>
-      <c r="W90" s="7">
+      <c r="V90" s="6"/>
+      <c r="W90" s="6">
         <v>-1.6630730581278801</v>
       </c>
-      <c r="X90" s="7"/>
-      <c r="Y90" s="7">
+      <c r="X90" s="6"/>
+      <c r="Y90" s="6">
         <v>-1.7136387929656201</v>
       </c>
     </row>
@@ -7691,80 +7785,80 @@
         <v>-13.0876453054645</v>
       </c>
     </row>
-    <row r="96" spans="1:25" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A96" s="7" t="s">
+    <row r="96" spans="1:25" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A96" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B96" s="7" t="s">
+      <c r="B96" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C96" s="7" t="s">
+      <c r="C96" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D96" s="7" t="s">
+      <c r="D96" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="E96" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="F96" s="7" t="s">
+      <c r="E96" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F96" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="G96" s="7" t="s">
+      <c r="G96" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="H96" s="7" t="s">
+      <c r="H96" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="I96" s="7">
-        <v>0</v>
-      </c>
-      <c r="J96" s="7">
-        <v>0</v>
-      </c>
-      <c r="K96" s="7">
-        <v>0</v>
-      </c>
-      <c r="L96" s="7">
+      <c r="I96" s="6">
+        <v>0</v>
+      </c>
+      <c r="J96" s="6">
+        <v>0</v>
+      </c>
+      <c r="K96" s="6">
+        <v>0</v>
+      </c>
+      <c r="L96" s="6">
         <v>-0.102415747464111</v>
       </c>
-      <c r="M96" s="7">
+      <c r="M96" s="6">
         <v>-0.24728363450511701</v>
       </c>
-      <c r="N96" s="7">
+      <c r="N96" s="6">
         <v>-0.75124324037055001</v>
       </c>
-      <c r="O96" s="7">
+      <c r="O96" s="6">
         <v>-1.4615006462561999</v>
       </c>
-      <c r="P96" s="7">
+      <c r="P96" s="6">
         <v>-2.8429700069803299</v>
       </c>
-      <c r="Q96" s="7">
+      <c r="Q96" s="6">
         <v>-3.2864801424826799</v>
       </c>
-      <c r="R96" s="7">
+      <c r="R96" s="6">
         <v>-3.6109363962888099</v>
       </c>
-      <c r="S96" s="7">
+      <c r="S96" s="6">
         <v>-3.8221034641243801</v>
       </c>
-      <c r="T96" s="7">
+      <c r="T96" s="6">
         <v>-4.0003689603371901</v>
       </c>
-      <c r="U96" s="7">
+      <c r="U96" s="6">
         <v>-4.1228110113523799</v>
       </c>
-      <c r="V96" s="7">
+      <c r="V96" s="6">
         <v>-4.2209087787319</v>
       </c>
-      <c r="W96" s="7">
+      <c r="W96" s="6">
         <v>-4.3126731548522201</v>
       </c>
-      <c r="X96" s="7">
+      <c r="X96" s="6">
         <v>-4.3203175334207504</v>
       </c>
-      <c r="Y96" s="7">
+      <c r="Y96" s="6">
         <v>-4.3852291596764399</v>
       </c>
     </row>
@@ -9077,80 +9171,80 @@
         <v>-18.404075921453799</v>
       </c>
     </row>
-    <row r="114" spans="1:25" s="13" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A114" s="12" t="s">
+    <row r="114" spans="1:25" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A114" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B114" s="13" t="s">
+      <c r="B114" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="C114" s="13" t="s">
+      <c r="C114" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="D114" s="13" t="s">
+      <c r="D114" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="E114" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="F114" s="13" t="s">
+      <c r="E114" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F114" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="G114" s="13" t="s">
+      <c r="G114" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="H114" s="13" t="s">
+      <c r="H114" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="I114" s="13">
+      <c r="I114" s="12">
         <v>-1.1414794825145901E-3</v>
       </c>
-      <c r="J114" s="13">
+      <c r="J114" s="12">
         <v>-6.8947149302056295E-4</v>
       </c>
-      <c r="K114" s="13">
+      <c r="K114" s="12">
         <v>-1.5552674895052201</v>
       </c>
-      <c r="L114" s="13">
+      <c r="L114" s="12">
         <v>-1.8161790686524999</v>
       </c>
-      <c r="M114" s="13">
+      <c r="M114" s="12">
         <v>-0.67370809182092795</v>
       </c>
-      <c r="N114" s="13">
+      <c r="N114" s="12">
         <v>-1.92936941876517</v>
       </c>
-      <c r="O114" s="10">
+      <c r="O114" s="9">
         <v>-2.5922501133826898</v>
       </c>
-      <c r="P114" s="13">
+      <c r="P114" s="12">
         <v>-4.30593661226861</v>
       </c>
-      <c r="Q114" s="13">
+      <c r="Q114" s="12">
         <v>-4.7479747573069</v>
       </c>
-      <c r="R114" s="13">
+      <c r="R114" s="12">
         <v>-5.935079002108</v>
       </c>
-      <c r="S114" s="13">
+      <c r="S114" s="12">
         <v>-8.0812599591154104</v>
       </c>
-      <c r="T114" s="11">
+      <c r="T114" s="10">
         <v>-9.8824917615499004</v>
       </c>
-      <c r="U114" s="13">
+      <c r="U114" s="12">
         <v>-7.2572785194595797</v>
       </c>
-      <c r="V114" s="13">
+      <c r="V114" s="12">
         <v>-9.4716694173467904</v>
       </c>
-      <c r="W114" s="13">
+      <c r="W114" s="12">
         <v>-8.8730556926694906</v>
       </c>
-      <c r="X114" s="13">
+      <c r="X114" s="12">
         <v>-8.0433965781073304</v>
       </c>
-      <c r="Y114" s="10">
+      <c r="Y114" s="9">
         <v>-6.6012693563680997</v>
       </c>
     </row>
@@ -10925,80 +11019,80 @@
         <v>-42.026492424003699</v>
       </c>
     </row>
-    <row r="138" spans="1:25" s="13" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A138" s="12" t="s">
+    <row r="138" spans="1:25" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A138" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B138" s="13" t="s">
+      <c r="B138" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="C138" s="13" t="s">
+      <c r="C138" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="D138" s="13" t="s">
+      <c r="D138" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="E138" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="F138" s="13" t="s">
+      <c r="E138" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F138" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="G138" s="13" t="s">
+      <c r="G138" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="H138" s="13" t="s">
+      <c r="H138" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="I138" s="13">
+      <c r="I138" s="12">
         <v>-8.3744962497281404E-4</v>
       </c>
-      <c r="J138" s="13">
+      <c r="J138" s="12">
         <v>-3.3871153074417002E-4</v>
       </c>
-      <c r="K138" s="13">
+      <c r="K138" s="12">
         <v>-1.37395219424134</v>
       </c>
-      <c r="L138" s="13">
+      <c r="L138" s="12">
         <v>-6.1642199949538803</v>
       </c>
-      <c r="M138" s="13">
+      <c r="M138" s="12">
         <v>-3.23103853522852</v>
       </c>
-      <c r="N138" s="13">
+      <c r="N138" s="12">
         <v>-4.5586636656420101</v>
       </c>
-      <c r="O138" s="10">
+      <c r="O138" s="9">
         <v>-5.6174259206717103</v>
       </c>
-      <c r="P138" s="13">
+      <c r="P138" s="12">
         <v>-9.1006329281160294</v>
       </c>
-      <c r="Q138" s="11">
+      <c r="Q138" s="10">
         <v>-10.8657006990382</v>
       </c>
-      <c r="R138" s="13">
+      <c r="R138" s="12">
         <v>-9.2734638751549401</v>
       </c>
-      <c r="S138" s="13">
+      <c r="S138" s="12">
         <v>-7.91290039276294</v>
       </c>
-      <c r="T138" s="13">
+      <c r="T138" s="12">
         <v>-8.7132243484834806</v>
       </c>
-      <c r="U138" s="13">
+      <c r="U138" s="12">
         <v>-8.3844226356329195</v>
       </c>
-      <c r="V138" s="13">
+      <c r="V138" s="12">
         <v>-7.8884772895334896</v>
       </c>
-      <c r="W138" s="13">
+      <c r="W138" s="12">
         <v>-7.84700241930177</v>
       </c>
-      <c r="X138" s="13">
+      <c r="X138" s="12">
         <v>-7.8349903602626902</v>
       </c>
-      <c r="Y138" s="10">
+      <c r="Y138" s="9">
         <v>-7.5999651473051104</v>
       </c>
     </row>
@@ -13515,4 +13609,1631 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4612D9FE-0ED7-4B4D-9D8C-D3A2173C3CAC}">
+  <dimension ref="A1:Y21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="18" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A2" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="H2" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="I2" s="17">
+        <v>0</v>
+      </c>
+      <c r="J2" s="17">
+        <v>0</v>
+      </c>
+      <c r="K2" s="17">
+        <v>47.946399999999997</v>
+      </c>
+      <c r="L2" s="17">
+        <v>134.94569999999999</v>
+      </c>
+      <c r="M2" s="17">
+        <v>180.49539999999999</v>
+      </c>
+      <c r="N2" s="17">
+        <v>221.3169</v>
+      </c>
+      <c r="O2" s="19">
+        <v>298.34769999999997</v>
+      </c>
+      <c r="P2" s="17">
+        <v>689.84519999999998</v>
+      </c>
+      <c r="Q2" s="17">
+        <v>704.44669999999996</v>
+      </c>
+      <c r="R2" s="17">
+        <v>129.45959999999999</v>
+      </c>
+      <c r="S2" s="17">
+        <v>229.04589999999999</v>
+      </c>
+      <c r="T2" s="17">
+        <v>297.38600000000002</v>
+      </c>
+      <c r="U2" s="17">
+        <v>302.98630000000003</v>
+      </c>
+      <c r="V2" s="17">
+        <v>294.05889999999999</v>
+      </c>
+      <c r="W2" s="17">
+        <v>329.9556</v>
+      </c>
+      <c r="X2" s="17">
+        <v>478.77480000000003</v>
+      </c>
+      <c r="Y2" s="19">
+        <v>648.00639999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A3" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="H3" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="I3" s="17">
+        <v>0</v>
+      </c>
+      <c r="J3" s="17">
+        <v>0</v>
+      </c>
+      <c r="K3" s="17">
+        <v>75.0715</v>
+      </c>
+      <c r="L3" s="17">
+        <v>107.4808</v>
+      </c>
+      <c r="M3" s="17">
+        <v>70.038899999999998</v>
+      </c>
+      <c r="N3" s="17">
+        <v>91.084100000000007</v>
+      </c>
+      <c r="O3" s="19">
+        <v>119.52760000000001</v>
+      </c>
+      <c r="P3" s="17">
+        <v>211.18879999999999</v>
+      </c>
+      <c r="Q3" s="17">
+        <v>274.69099999999997</v>
+      </c>
+      <c r="R3" s="17">
+        <v>352.67910000000001</v>
+      </c>
+      <c r="S3" s="17">
+        <v>549.74680000000001</v>
+      </c>
+      <c r="T3" s="17">
+        <v>716.22850000000005</v>
+      </c>
+      <c r="U3" s="17">
+        <v>342.47489999999999</v>
+      </c>
+      <c r="V3" s="17">
+        <v>718.26859999999999</v>
+      </c>
+      <c r="W3" s="17">
+        <v>719.8664</v>
+      </c>
+      <c r="X3" s="17">
+        <v>713.50340000000006</v>
+      </c>
+      <c r="Y3" s="19">
+        <v>536.79160000000002</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A4" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H4" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="I4" s="17">
+        <v>0</v>
+      </c>
+      <c r="J4" s="17">
+        <v>0</v>
+      </c>
+      <c r="K4" s="17">
+        <v>5.5458999999999996</v>
+      </c>
+      <c r="L4" s="17">
+        <v>4.9405000000000001</v>
+      </c>
+      <c r="M4" s="17">
+        <v>71.909400000000005</v>
+      </c>
+      <c r="N4" s="17">
+        <v>107.1816</v>
+      </c>
+      <c r="O4" s="19">
+        <v>144.29230000000001</v>
+      </c>
+      <c r="P4" s="17">
+        <v>202.06010000000001</v>
+      </c>
+      <c r="Q4" s="17">
+        <v>322.90879999999999</v>
+      </c>
+      <c r="R4" s="17">
+        <v>593.98360000000002</v>
+      </c>
+      <c r="S4" s="17">
+        <v>713.03250000000003</v>
+      </c>
+      <c r="T4" s="17">
+        <v>716.11850000000004</v>
+      </c>
+      <c r="U4" s="17">
+        <v>773.36220000000003</v>
+      </c>
+      <c r="V4" s="17">
+        <v>805.63239999999996</v>
+      </c>
+      <c r="W4" s="17">
+        <v>716.91589999999997</v>
+      </c>
+      <c r="X4" s="17">
+        <v>714.26390000000004</v>
+      </c>
+      <c r="Y4" s="19">
+        <v>718.51279999999997</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A5" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H5" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="I5" s="17">
+        <v>0</v>
+      </c>
+      <c r="J5" s="17">
+        <v>0</v>
+      </c>
+      <c r="K5" s="17">
+        <v>8.7279999999999998</v>
+      </c>
+      <c r="L5" s="17">
+        <v>8.7279999999999998</v>
+      </c>
+      <c r="M5" s="17">
+        <v>8.7279999999999998</v>
+      </c>
+      <c r="N5" s="17">
+        <v>8.7279999999999998</v>
+      </c>
+      <c r="O5" s="19">
+        <v>8.7279999999999998</v>
+      </c>
+      <c r="P5" s="17">
+        <v>8.7279999999999998</v>
+      </c>
+      <c r="Q5" s="17">
+        <v>8.7279999999999998</v>
+      </c>
+      <c r="R5" s="17">
+        <v>8.7279999999999998</v>
+      </c>
+      <c r="S5" s="17">
+        <v>8.7279999999999998</v>
+      </c>
+      <c r="T5" s="17">
+        <v>8.7279999999999998</v>
+      </c>
+      <c r="U5" s="17">
+        <v>8.7279999999999998</v>
+      </c>
+      <c r="V5" s="17">
+        <v>8.7279999999999998</v>
+      </c>
+      <c r="W5" s="17">
+        <v>8.7279999999999998</v>
+      </c>
+      <c r="X5" s="17">
+        <v>8.7279999999999998</v>
+      </c>
+      <c r="Y5" s="19">
+        <v>8.7279999999999998</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A6" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="H6" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6" s="17">
+        <v>0</v>
+      </c>
+      <c r="J6" s="17">
+        <v>0</v>
+      </c>
+      <c r="K6" s="17">
+        <v>1</v>
+      </c>
+      <c r="L6" s="17">
+        <v>1</v>
+      </c>
+      <c r="M6" s="17">
+        <v>1</v>
+      </c>
+      <c r="N6" s="17">
+        <v>1</v>
+      </c>
+      <c r="O6" s="19">
+        <v>1</v>
+      </c>
+      <c r="P6" s="17">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="17">
+        <v>20.629100000000001</v>
+      </c>
+      <c r="R6" s="17">
+        <v>78.445300000000003</v>
+      </c>
+      <c r="S6" s="17">
+        <v>129.9402</v>
+      </c>
+      <c r="T6" s="17">
+        <v>178.56649999999999</v>
+      </c>
+      <c r="U6" s="17">
+        <v>260.57740000000001</v>
+      </c>
+      <c r="V6" s="17">
+        <v>445.05849999999998</v>
+      </c>
+      <c r="W6" s="17">
+        <v>475.16149999999999</v>
+      </c>
+      <c r="X6" s="17">
+        <v>210.6396</v>
+      </c>
+      <c r="Y6" s="19">
+        <v>272.30439999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A7" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="G7" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="I7" s="17">
+        <v>0</v>
+      </c>
+      <c r="J7" s="17">
+        <v>0</v>
+      </c>
+      <c r="K7" s="17">
+        <v>95.398200000000003</v>
+      </c>
+      <c r="L7" s="17">
+        <v>317.68849999999998</v>
+      </c>
+      <c r="M7" s="17">
+        <v>249.05350000000001</v>
+      </c>
+      <c r="N7" s="17">
+        <v>233.00200000000001</v>
+      </c>
+      <c r="O7" s="19">
+        <v>239.9537</v>
+      </c>
+      <c r="P7" s="17">
+        <v>322.43090000000001</v>
+      </c>
+      <c r="Q7" s="17">
+        <v>713.2998</v>
+      </c>
+      <c r="R7" s="17">
+        <v>612.39329999999995</v>
+      </c>
+      <c r="S7" s="17">
+        <v>347.79160000000002</v>
+      </c>
+      <c r="T7" s="17">
+        <v>386.84460000000001</v>
+      </c>
+      <c r="U7" s="17">
+        <v>395.97320000000002</v>
+      </c>
+      <c r="V7" s="17">
+        <v>395.79469999999998</v>
+      </c>
+      <c r="W7" s="17">
+        <v>415.34249999999997</v>
+      </c>
+      <c r="X7" s="17">
+        <v>435.02510000000001</v>
+      </c>
+      <c r="Y7" s="19">
+        <v>385.73090000000002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" t="s">
+        <v>66</v>
+      </c>
+      <c r="E8" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" t="s">
+        <v>55</v>
+      </c>
+      <c r="H8" t="s">
+        <v>32</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
+      <c r="N8">
+        <v>0</v>
+      </c>
+      <c r="O8" s="18">
+        <v>0</v>
+      </c>
+      <c r="P8">
+        <v>0</v>
+      </c>
+      <c r="Q8">
+        <v>0</v>
+      </c>
+      <c r="R8">
+        <v>0</v>
+      </c>
+      <c r="S8">
+        <v>0</v>
+      </c>
+      <c r="T8">
+        <v>0</v>
+      </c>
+      <c r="U8">
+        <v>0</v>
+      </c>
+      <c r="V8">
+        <v>0</v>
+      </c>
+      <c r="W8">
+        <v>0</v>
+      </c>
+      <c r="X8">
+        <v>0</v>
+      </c>
+      <c r="Y8" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="I9" s="12">
+        <v>-1.0578632109699501E-3</v>
+      </c>
+      <c r="J9" s="12">
+        <v>4.1697844225231602E-2</v>
+      </c>
+      <c r="K9" s="12">
+        <v>-0.16286460592993199</v>
+      </c>
+      <c r="L9" s="12">
+        <v>-1.1605026255561699</v>
+      </c>
+      <c r="M9" s="12">
+        <v>-2.1262221245153898</v>
+      </c>
+      <c r="N9" s="12">
+        <v>-2.9890608058457002</v>
+      </c>
+      <c r="O9" s="20">
+        <v>-3.81855918047148</v>
+      </c>
+      <c r="P9" s="10">
+        <v>-5.3700453030046997</v>
+      </c>
+      <c r="Q9" s="12">
+        <v>-4.9159529147579102</v>
+      </c>
+      <c r="R9" s="12">
+        <v>-2.9293700720396498</v>
+      </c>
+      <c r="S9" s="12">
+        <v>-3.0956558169340598</v>
+      </c>
+      <c r="T9" s="12">
+        <v>-3.14404581467184</v>
+      </c>
+      <c r="U9" s="12">
+        <v>-3.09084100825834</v>
+      </c>
+      <c r="V9" s="12">
+        <v>-2.9612883223045898</v>
+      </c>
+      <c r="W9" s="12">
+        <v>-2.9780504314503302</v>
+      </c>
+      <c r="X9" s="12">
+        <v>-3.3179844014514601</v>
+      </c>
+      <c r="Y9" s="20">
+        <v>-3.5920532046805902</v>
+      </c>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A10" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="E10" s="29" t="s">
+        <v>54</v>
+      </c>
+      <c r="F10" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="G10" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="H10" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="I10" s="29">
+        <v>-8.7913750073166999E-4</v>
+      </c>
+      <c r="J10" s="29">
+        <v>-5.8332650511705799E-4</v>
+      </c>
+      <c r="K10" s="29">
+        <v>-0.36260718770109401</v>
+      </c>
+      <c r="L10" s="29">
+        <v>-0.70973931104547405</v>
+      </c>
+      <c r="M10" s="29">
+        <v>-0.46387274310988502</v>
+      </c>
+      <c r="N10" s="29">
+        <v>-1.0911267095544599</v>
+      </c>
+      <c r="O10" s="30">
+        <v>-1.6434290536272</v>
+      </c>
+      <c r="P10" s="29">
+        <v>-2.4881449937226998</v>
+      </c>
+      <c r="Q10" s="29">
+        <v>-3.1756219186050401</v>
+      </c>
+      <c r="R10" s="29">
+        <v>-3.7951404595943199</v>
+      </c>
+      <c r="S10" s="29">
+        <v>-4.9206087414089499</v>
+      </c>
+      <c r="T10" s="31">
+        <v>-5.3157227290386002</v>
+      </c>
+      <c r="U10" s="29">
+        <v>-4.0423714719693598</v>
+      </c>
+      <c r="V10" s="29">
+        <v>-5.2003308370125598</v>
+      </c>
+      <c r="W10" s="29">
+        <v>-4.7058093442706799</v>
+      </c>
+      <c r="X10" s="29">
+        <v>-4.3698814438566904</v>
+      </c>
+      <c r="Y10" s="32">
+        <v>-3.7840036088050302</v>
+      </c>
+    </row>
+    <row r="11" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I11" s="1">
+        <v>-9.0744916322244604E-4</v>
+      </c>
+      <c r="J11" s="1">
+        <v>-7.1042955919197598E-4</v>
+      </c>
+      <c r="K11" s="1">
+        <v>1.2529108917522999E-2</v>
+      </c>
+      <c r="L11" s="1">
+        <v>-1.9526940536319301E-2</v>
+      </c>
+      <c r="M11" s="1">
+        <v>-1.15752168185981</v>
+      </c>
+      <c r="N11" s="1">
+        <v>-1.62046275476018</v>
+      </c>
+      <c r="O11" s="18">
+        <v>-2.2231122989782399</v>
+      </c>
+      <c r="P11" s="1">
+        <v>-2.96943218925245</v>
+      </c>
+      <c r="Q11" s="1">
+        <v>-3.8372615607490101</v>
+      </c>
+      <c r="R11" s="1">
+        <v>-5.0875278150906302</v>
+      </c>
+      <c r="S11" s="2">
+        <v>-5.5103782824654504</v>
+      </c>
+      <c r="T11" s="2">
+        <v>-5.5242883117707304</v>
+      </c>
+      <c r="U11" s="1">
+        <v>-4.95848716923601</v>
+      </c>
+      <c r="V11" s="1">
+        <v>-3.7284877182373402</v>
+      </c>
+      <c r="W11" s="1">
+        <v>-2.8740632738956702</v>
+      </c>
+      <c r="X11" s="1">
+        <v>-3.0361906524501898</v>
+      </c>
+      <c r="Y11" s="18">
+        <v>-3.0219728536580202</v>
+      </c>
+    </row>
+    <row r="12" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" t="s">
+        <v>66</v>
+      </c>
+      <c r="E12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F12" t="s">
+        <v>34</v>
+      </c>
+      <c r="G12" t="s">
+        <v>39</v>
+      </c>
+      <c r="H12" t="s">
+        <v>32</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>0</v>
+      </c>
+      <c r="N12">
+        <v>0</v>
+      </c>
+      <c r="O12" s="18">
+        <v>0</v>
+      </c>
+      <c r="P12">
+        <v>0</v>
+      </c>
+      <c r="Q12">
+        <v>0</v>
+      </c>
+      <c r="R12">
+        <v>0</v>
+      </c>
+      <c r="S12">
+        <v>0</v>
+      </c>
+      <c r="T12">
+        <v>0</v>
+      </c>
+      <c r="U12">
+        <v>0</v>
+      </c>
+      <c r="V12">
+        <v>0</v>
+      </c>
+      <c r="W12">
+        <v>0</v>
+      </c>
+      <c r="X12">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" t="s">
+        <v>66</v>
+      </c>
+      <c r="E13" t="s">
+        <v>54</v>
+      </c>
+      <c r="F13" t="s">
+        <v>34</v>
+      </c>
+      <c r="G13" t="s">
+        <v>41</v>
+      </c>
+      <c r="H13" t="s">
+        <v>32</v>
+      </c>
+      <c r="I13">
+        <v>-4.8116408388063601E-4</v>
+      </c>
+      <c r="J13">
+        <v>6.5778399950188805E-5</v>
+      </c>
+      <c r="K13">
+        <v>4.4460659212569198E-2</v>
+      </c>
+      <c r="L13">
+        <v>2.2152483096230598E-3</v>
+      </c>
+      <c r="M13">
+        <v>-2.6005910209274299E-2</v>
+      </c>
+      <c r="N13">
+        <v>-3.2841559460654299E-2</v>
+      </c>
+      <c r="O13" s="18">
+        <v>-5.7055621910321798E-2</v>
+      </c>
+      <c r="P13">
+        <v>-4.3408051781953901E-2</v>
+      </c>
+      <c r="Q13">
+        <v>-0.354280079858458</v>
+      </c>
+      <c r="R13">
+        <v>-1.0129346962212</v>
+      </c>
+      <c r="S13">
+        <v>-1.6859498767372101</v>
+      </c>
+      <c r="T13">
+        <v>-2.3255091075405199</v>
+      </c>
+      <c r="U13">
+        <v>-3.15034260913029</v>
+      </c>
+      <c r="V13">
+        <v>-3.9500565454043302</v>
+      </c>
+      <c r="W13">
+        <v>-3.9622315664754701</v>
+      </c>
+      <c r="X13">
+        <v>-3.01483067186612</v>
+      </c>
+      <c r="Y13" s="18">
+        <v>-3.3281006635520902</v>
+      </c>
+    </row>
+    <row r="14" spans="1:25" s="23" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="23" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="E14" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="G14" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="H14" s="23" t="s">
+        <v>32</v>
+      </c>
+      <c r="I14" s="23">
+        <v>-6.4526438354928402E-4</v>
+      </c>
+      <c r="J14" s="23">
+        <v>-2.8138537756838898E-4</v>
+      </c>
+      <c r="K14" s="23">
+        <v>-0.18662432866873499</v>
+      </c>
+      <c r="L14" s="23">
+        <v>-2.2820558133245901</v>
+      </c>
+      <c r="M14" s="23">
+        <v>-2.0152449032145299</v>
+      </c>
+      <c r="N14" s="23">
+        <v>-2.9417147205340601</v>
+      </c>
+      <c r="O14" s="24">
+        <v>-3.5465996387186798</v>
+      </c>
+      <c r="P14" s="23">
+        <v>-4.8331370562782396</v>
+      </c>
+      <c r="Q14" s="25">
+        <v>-6.4120026541508004</v>
+      </c>
+      <c r="R14" s="23">
+        <v>-5.8685094717820796</v>
+      </c>
+      <c r="S14" s="23">
+        <v>-4.97600469012826</v>
+      </c>
+      <c r="T14" s="23">
+        <v>-5.1867705410924403</v>
+      </c>
+      <c r="U14" s="23">
+        <v>-5.1431987307323697</v>
+      </c>
+      <c r="V14" s="23">
+        <v>-5.1449302502717504</v>
+      </c>
+      <c r="W14" s="23">
+        <v>-5.1915414749731097</v>
+      </c>
+      <c r="X14" s="23">
+        <v>-5.2318674913929</v>
+      </c>
+      <c r="Y14" s="24">
+        <v>-5.14824197838725</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A15" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="G15" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="H15" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="I15" s="13">
+        <v>0</v>
+      </c>
+      <c r="J15" s="13">
+        <v>0</v>
+      </c>
+      <c r="K15" s="13">
+        <v>0</v>
+      </c>
+      <c r="L15" s="13">
+        <v>0</v>
+      </c>
+      <c r="M15" s="13">
+        <v>0</v>
+      </c>
+      <c r="N15" s="13">
+        <v>0</v>
+      </c>
+      <c r="O15" s="21">
+        <v>0</v>
+      </c>
+      <c r="P15" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="13">
+        <v>0</v>
+      </c>
+      <c r="R15" s="13">
+        <v>0</v>
+      </c>
+      <c r="S15" s="13">
+        <v>0</v>
+      </c>
+      <c r="T15" s="13">
+        <v>0</v>
+      </c>
+      <c r="U15" s="13">
+        <v>0</v>
+      </c>
+      <c r="V15" s="13">
+        <v>0</v>
+      </c>
+      <c r="W15" s="13">
+        <v>0</v>
+      </c>
+      <c r="X15" s="13">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="F16" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="G16" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="H16" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="I16" s="15">
+        <v>-1.40121687066601E-3</v>
+      </c>
+      <c r="J16" s="15">
+        <v>2.9810544407359099E-2</v>
+      </c>
+      <c r="K16" s="15">
+        <v>-1.00497740230282</v>
+      </c>
+      <c r="L16" s="15">
+        <v>-2.8730061124521802</v>
+      </c>
+      <c r="M16" s="15">
+        <v>-3.3915688163490501</v>
+      </c>
+      <c r="N16" s="15">
+        <v>-4.2934834435993903</v>
+      </c>
+      <c r="O16" s="22">
+        <v>-5.5240503558825802</v>
+      </c>
+      <c r="P16" s="15">
+        <v>-9.3763703767265607</v>
+      </c>
+      <c r="Q16" s="15">
+        <v>-8.4269242283516395</v>
+      </c>
+      <c r="R16" s="15">
+        <v>-5.36160514363233</v>
+      </c>
+      <c r="S16" s="15">
+        <v>-5.4422016956287598</v>
+      </c>
+      <c r="T16" s="15">
+        <v>-5.9187732047331298</v>
+      </c>
+      <c r="U16" s="15">
+        <v>-5.3131350881682904</v>
+      </c>
+      <c r="V16" s="15">
+        <v>-4.8096068076143501</v>
+      </c>
+      <c r="W16" s="15">
+        <v>-4.8861347792670999</v>
+      </c>
+      <c r="X16" s="15">
+        <v>-5.5496521996296204</v>
+      </c>
+      <c r="Y16" s="22">
+        <v>-5.9697097227904399</v>
+      </c>
+    </row>
+    <row r="17" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A17" s="33" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" s="34" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="34" t="s">
+        <v>67</v>
+      </c>
+      <c r="E17" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="F17" s="34" t="s">
+        <v>34</v>
+      </c>
+      <c r="G17" s="34" t="s">
+        <v>35</v>
+      </c>
+      <c r="H17" s="34" t="s">
+        <v>32</v>
+      </c>
+      <c r="I17" s="34">
+        <v>-1.1414794825145901E-3</v>
+      </c>
+      <c r="J17" s="34">
+        <v>-6.8947149302056295E-4</v>
+      </c>
+      <c r="K17" s="34">
+        <v>-1.5552674895052201</v>
+      </c>
+      <c r="L17" s="34">
+        <v>-1.8161790686524999</v>
+      </c>
+      <c r="M17" s="34">
+        <v>-0.67370809182092795</v>
+      </c>
+      <c r="N17" s="34">
+        <v>-1.92936941876517</v>
+      </c>
+      <c r="O17" s="35">
+        <v>-2.5922501133826898</v>
+      </c>
+      <c r="P17" s="34">
+        <v>-4.30593661226861</v>
+      </c>
+      <c r="Q17" s="34">
+        <v>-4.7479747573069</v>
+      </c>
+      <c r="R17" s="34">
+        <v>-5.935079002108</v>
+      </c>
+      <c r="S17" s="34">
+        <v>-8.0812599591154104</v>
+      </c>
+      <c r="T17" s="34">
+        <v>-9.8824917615499004</v>
+      </c>
+      <c r="U17" s="34">
+        <v>-7.2572785194595797</v>
+      </c>
+      <c r="V17" s="34">
+        <v>-9.4716694173467904</v>
+      </c>
+      <c r="W17" s="34">
+        <v>-8.8730556926694906</v>
+      </c>
+      <c r="X17" s="34">
+        <v>-8.0433965781073304</v>
+      </c>
+      <c r="Y17" s="36">
+        <v>-6.6012693563680997</v>
+      </c>
+    </row>
+    <row r="18" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A18" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="D18" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="E18" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="F18" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="G18" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="H18" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="I18" s="16">
+        <v>-1.1907100862477099E-3</v>
+      </c>
+      <c r="J18" s="16">
+        <v>-8.9022848302213603E-4</v>
+      </c>
+      <c r="K18" s="16">
+        <v>8.7775015733854798E-3</v>
+      </c>
+      <c r="L18" s="16">
+        <v>3.8006556644464701E-2</v>
+      </c>
+      <c r="M18" s="16">
+        <v>-2.7996730918756798</v>
+      </c>
+      <c r="N18" s="16">
+        <v>-2.5049776614694399</v>
+      </c>
+      <c r="O18" s="21">
+        <v>-3.3990333066364999</v>
+      </c>
+      <c r="P18" s="16">
+        <v>-4.8014595627444701</v>
+      </c>
+      <c r="Q18" s="16">
+        <v>-6.4964035963353099</v>
+      </c>
+      <c r="R18" s="16">
+        <v>-8.6286655405999095</v>
+      </c>
+      <c r="S18" s="16">
+        <v>-9.7191816012847898</v>
+      </c>
+      <c r="T18" s="16">
+        <v>-10.2269000231219</v>
+      </c>
+      <c r="U18" s="16">
+        <v>-12.3759995272694</v>
+      </c>
+      <c r="V18" s="16">
+        <v>-11.9255379919046</v>
+      </c>
+      <c r="W18" s="16">
+        <v>-9.8163342476181494</v>
+      </c>
+      <c r="X18" s="16">
+        <v>-9.5449152977915794</v>
+      </c>
+      <c r="Y18" s="21">
+        <v>-10.1987077771962</v>
+      </c>
+    </row>
+    <row r="19" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A19" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="G19" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="H19" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="I19" s="13">
+        <v>0</v>
+      </c>
+      <c r="J19" s="13">
+        <v>0</v>
+      </c>
+      <c r="K19" s="13">
+        <v>0</v>
+      </c>
+      <c r="L19" s="13">
+        <v>0</v>
+      </c>
+      <c r="M19" s="13">
+        <v>0</v>
+      </c>
+      <c r="N19" s="13">
+        <v>0</v>
+      </c>
+      <c r="O19" s="21">
+        <v>0</v>
+      </c>
+      <c r="P19" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="13">
+        <v>0</v>
+      </c>
+      <c r="R19" s="13">
+        <v>0</v>
+      </c>
+      <c r="S19" s="13">
+        <v>0</v>
+      </c>
+      <c r="T19" s="13">
+        <v>0</v>
+      </c>
+      <c r="U19" s="13">
+        <v>0</v>
+      </c>
+      <c r="V19" s="13">
+        <v>0</v>
+      </c>
+      <c r="W19" s="13">
+        <v>0</v>
+      </c>
+      <c r="X19" s="13">
+        <v>0</v>
+      </c>
+      <c r="Y19" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A20" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="G20" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="H20" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="I20" s="13">
+        <v>-6.4440919309741098E-4</v>
+      </c>
+      <c r="J20" s="13">
+        <v>8.2381150446786305E-5</v>
+      </c>
+      <c r="K20" s="13">
+        <v>0.20369528686966201</v>
+      </c>
+      <c r="L20" s="13">
+        <v>8.9490252552921007E-2</v>
+      </c>
+      <c r="M20" s="13">
+        <v>5.14537535944092E-2</v>
+      </c>
+      <c r="N20" s="13">
+        <v>-1.13484060300529E-2</v>
+      </c>
+      <c r="O20" s="21">
+        <v>9.9966013764362094E-3</v>
+      </c>
+      <c r="P20" s="13">
+        <v>-1.86021197951864E-2</v>
+      </c>
+      <c r="Q20" s="13">
+        <v>-0.52891915560452196</v>
+      </c>
+      <c r="R20" s="13">
+        <v>-1.69887278576212</v>
+      </c>
+      <c r="S20" s="13">
+        <v>-2.5030760354409698</v>
+      </c>
+      <c r="T20" s="13">
+        <v>-3.5565076202561099</v>
+      </c>
+      <c r="U20" s="13">
+        <v>-4.70718181881041</v>
+      </c>
+      <c r="V20" s="13">
+        <v>-6.3974527845875198</v>
+      </c>
+      <c r="W20" s="13">
+        <v>-6.1986554630048598</v>
+      </c>
+      <c r="X20" s="13">
+        <v>-4.5925798877115502</v>
+      </c>
+      <c r="Y20" s="21">
+        <v>-4.9005807954648697</v>
+      </c>
+    </row>
+    <row r="21" spans="1:25" s="23" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" s="26" t="s">
+        <v>27</v>
+      </c>
+      <c r="D21" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="E21" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="F21" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="G21" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="H21" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="I21" s="26">
+        <v>-8.3744962497281404E-4</v>
+      </c>
+      <c r="J21" s="26">
+        <v>-3.3871153074417002E-4</v>
+      </c>
+      <c r="K21" s="26">
+        <v>-1.37395219424134</v>
+      </c>
+      <c r="L21" s="26">
+        <v>-6.1642199949538803</v>
+      </c>
+      <c r="M21" s="26">
+        <v>-3.23103853522852</v>
+      </c>
+      <c r="N21" s="26">
+        <v>-4.5586636656420101</v>
+      </c>
+      <c r="O21" s="27">
+        <v>-5.6174259206717103</v>
+      </c>
+      <c r="P21" s="26">
+        <v>-9.1006329281160294</v>
+      </c>
+      <c r="Q21" s="26">
+        <v>-10.8657006990382</v>
+      </c>
+      <c r="R21" s="26">
+        <v>-9.2734638751549401</v>
+      </c>
+      <c r="S21" s="26">
+        <v>-7.91290039276294</v>
+      </c>
+      <c r="T21" s="26">
+        <v>-8.7132243484834806</v>
+      </c>
+      <c r="U21" s="26">
+        <v>-8.3844226356329195</v>
+      </c>
+      <c r="V21" s="26">
+        <v>-7.8884772895334896</v>
+      </c>
+      <c r="W21" s="26">
+        <v>-7.84700241930177</v>
+      </c>
+      <c r="X21" s="26">
+        <v>-7.8349903602626902</v>
+      </c>
+      <c r="Y21" s="27">
+        <v>-7.5999651473051104</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>